<commit_message>
Add Sept Renewal Report view to dashboard and remove Distinguished Status Distribution chart from Overview
</commit_message>
<xml_diff>
--- a/District 121 - Mastersheet.xlsx
+++ b/District 121 - Mastersheet.xlsx
@@ -13015,7 +13015,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M190"/>
+  <dimension ref="A1:O190"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -13031,6 +13031,8 @@
     <col width="21" customWidth="1" min="11" max="11"/>
     <col width="17" customWidth="1" min="12" max="12"/>
     <col width="17" customWidth="1" min="13" max="13"/>
+    <col width="17" customWidth="1" min="14" max="14"/>
+    <col width="17" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -13099,6 +13101,16 @@
           <t>Total Payments</t>
         </is>
       </c>
+      <c r="N1" s="14" t="inlineStr">
+        <is>
+          <t>Single Renewal</t>
+        </is>
+      </c>
+      <c r="O1" s="14" t="inlineStr">
+        <is>
+          <t>Double Renewal</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="15" t="n">
@@ -13150,6 +13162,12 @@
       <c r="M2" s="17" t="n">
         <v>12</v>
       </c>
+      <c r="N2" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="O2" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="18" t="n">
@@ -13201,6 +13219,12 @@
       <c r="M3" s="20" t="n">
         <v>73</v>
       </c>
+      <c r="N3" s="20" t="n">
+        <v>25</v>
+      </c>
+      <c r="O3" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="15" t="n">
@@ -13252,6 +13276,12 @@
       <c r="M4" s="17" t="n">
         <v>56</v>
       </c>
+      <c r="N4" s="17" t="n">
+        <v>22</v>
+      </c>
+      <c r="O4" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="18" t="n">
@@ -13303,6 +13333,12 @@
       <c r="M5" s="20" t="n">
         <v>37</v>
       </c>
+      <c r="N5" s="20" t="n">
+        <v>11</v>
+      </c>
+      <c r="O5" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="15" t="n">
@@ -13354,6 +13390,12 @@
       <c r="M6" s="17" t="n">
         <v>52</v>
       </c>
+      <c r="N6" s="17" t="n">
+        <v>26</v>
+      </c>
+      <c r="O6" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="18" t="n">
@@ -13405,6 +13447,12 @@
       <c r="M7" s="20" t="n">
         <v>21</v>
       </c>
+      <c r="N7" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="O7" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="15" t="n">
@@ -13456,6 +13504,12 @@
       <c r="M8" s="17" t="n">
         <v>47</v>
       </c>
+      <c r="N8" s="17" t="n">
+        <v>13</v>
+      </c>
+      <c r="O8" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="18" t="n">
@@ -13507,6 +13561,12 @@
       <c r="M9" s="20" t="n">
         <v>77</v>
       </c>
+      <c r="N9" s="20" t="n">
+        <v>23</v>
+      </c>
+      <c r="O9" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="15" t="n">
@@ -13558,6 +13618,12 @@
       <c r="M10" s="17" t="n">
         <v>18</v>
       </c>
+      <c r="N10" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="O10" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="18" t="n">
@@ -13609,6 +13675,12 @@
       <c r="M11" s="20" t="n">
         <v>72</v>
       </c>
+      <c r="N11" s="20" t="n">
+        <v>9</v>
+      </c>
+      <c r="O11" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="15" t="n">
@@ -13660,6 +13732,12 @@
       <c r="M12" s="17" t="n">
         <v>19</v>
       </c>
+      <c r="N12" s="17" t="n">
+        <v>9</v>
+      </c>
+      <c r="O12" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="18" t="n">
@@ -13711,6 +13789,12 @@
       <c r="M13" s="20" t="n">
         <v>26</v>
       </c>
+      <c r="N13" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="O13" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="15" t="n">
@@ -13762,6 +13846,12 @@
       <c r="M14" s="17" t="n">
         <v>133</v>
       </c>
+      <c r="N14" s="17" t="n">
+        <v>59</v>
+      </c>
+      <c r="O14" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="18" t="n">
@@ -13813,6 +13903,12 @@
       <c r="M15" s="20" t="n">
         <v>72</v>
       </c>
+      <c r="N15" s="20" t="n">
+        <v>22</v>
+      </c>
+      <c r="O15" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="15" t="n">
@@ -13864,6 +13960,12 @@
       <c r="M16" s="17" t="n">
         <v>56</v>
       </c>
+      <c r="N16" s="17" t="n">
+        <v>14</v>
+      </c>
+      <c r="O16" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="18" t="n">
@@ -13915,6 +14017,12 @@
       <c r="M17" s="20" t="n">
         <v>0</v>
       </c>
+      <c r="N17" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="O17" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="15" t="n">
@@ -13966,6 +14074,12 @@
       <c r="M18" s="17" t="n">
         <v>40</v>
       </c>
+      <c r="N18" s="17" t="n">
+        <v>14</v>
+      </c>
+      <c r="O18" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="18" t="n">
@@ -14017,6 +14131,12 @@
       <c r="M19" s="20" t="n">
         <v>54</v>
       </c>
+      <c r="N19" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="O19" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="15" t="n">
@@ -14068,6 +14188,12 @@
       <c r="M20" s="17" t="n">
         <v>38</v>
       </c>
+      <c r="N20" s="17" t="n">
+        <v>15</v>
+      </c>
+      <c r="O20" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="18" t="n">
@@ -14119,6 +14245,12 @@
       <c r="M21" s="20" t="n">
         <v>50</v>
       </c>
+      <c r="N21" s="20" t="n">
+        <v>21</v>
+      </c>
+      <c r="O21" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="15" t="n">
@@ -14170,6 +14302,12 @@
       <c r="M22" s="17" t="n">
         <v>34</v>
       </c>
+      <c r="N22" s="17" t="n">
+        <v>14</v>
+      </c>
+      <c r="O22" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="18" t="n">
@@ -14221,6 +14359,12 @@
       <c r="M23" s="20" t="n">
         <v>47</v>
       </c>
+      <c r="N23" s="20" t="n">
+        <v>19</v>
+      </c>
+      <c r="O23" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="15" t="n">
@@ -14272,6 +14416,12 @@
       <c r="M24" s="17" t="n">
         <v>27</v>
       </c>
+      <c r="N24" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="O24" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="18" t="n">
@@ -14323,6 +14473,12 @@
       <c r="M25" s="20" t="n">
         <v>29</v>
       </c>
+      <c r="N25" s="20" t="n">
+        <v>14</v>
+      </c>
+      <c r="O25" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="15" t="n">
@@ -14374,6 +14530,12 @@
       <c r="M26" s="17" t="n">
         <v>27</v>
       </c>
+      <c r="N26" s="17" t="n">
+        <v>15</v>
+      </c>
+      <c r="O26" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="18" t="n">
@@ -14425,6 +14587,12 @@
       <c r="M27" s="20" t="n">
         <v>26</v>
       </c>
+      <c r="N27" s="20" t="n">
+        <v>16</v>
+      </c>
+      <c r="O27" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="15" t="n">
@@ -14476,6 +14644,12 @@
       <c r="M28" s="17" t="n">
         <v>28</v>
       </c>
+      <c r="N28" s="17" t="n">
+        <v>16</v>
+      </c>
+      <c r="O28" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="18" t="n">
@@ -14527,6 +14701,12 @@
       <c r="M29" s="20" t="n">
         <v>17</v>
       </c>
+      <c r="N29" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="O29" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="15" t="n">
@@ -14578,6 +14758,12 @@
       <c r="M30" s="17" t="n">
         <v>6</v>
       </c>
+      <c r="N30" s="17" t="n">
+        <v>5</v>
+      </c>
+      <c r="O30" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="18" t="n">
@@ -14629,6 +14815,12 @@
       <c r="M31" s="20" t="n">
         <v>165</v>
       </c>
+      <c r="N31" s="20" t="n">
+        <v>25</v>
+      </c>
+      <c r="O31" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="15" t="n">
@@ -14680,6 +14872,12 @@
       <c r="M32" s="17" t="n">
         <v>65</v>
       </c>
+      <c r="N32" s="17" t="n">
+        <v>18</v>
+      </c>
+      <c r="O32" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="18" t="n">
@@ -14731,6 +14929,12 @@
       <c r="M33" s="20" t="n">
         <v>20</v>
       </c>
+      <c r="N33" s="20" t="n">
+        <v>20</v>
+      </c>
+      <c r="O33" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="15" t="n">
@@ -14782,6 +14986,12 @@
       <c r="M34" s="17" t="n">
         <v>73</v>
       </c>
+      <c r="N34" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="O34" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="18" t="n">
@@ -14833,6 +15043,12 @@
       <c r="M35" s="20" t="n">
         <v>28</v>
       </c>
+      <c r="N35" s="20" t="n">
+        <v>12</v>
+      </c>
+      <c r="O35" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="15" t="n">
@@ -14884,6 +15100,12 @@
       <c r="M36" s="17" t="n">
         <v>41</v>
       </c>
+      <c r="N36" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="O36" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="18" t="n">
@@ -14935,6 +15157,12 @@
       <c r="M37" s="20" t="n">
         <v>33</v>
       </c>
+      <c r="N37" s="20" t="n">
+        <v>14</v>
+      </c>
+      <c r="O37" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="15" t="n">
@@ -14986,6 +15214,12 @@
       <c r="M38" s="17" t="n">
         <v>60</v>
       </c>
+      <c r="N38" s="17" t="n">
+        <v>26</v>
+      </c>
+      <c r="O38" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="18" t="n">
@@ -15037,6 +15271,12 @@
       <c r="M39" s="20" t="n">
         <v>0</v>
       </c>
+      <c r="N39" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="O39" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="15" t="n">
@@ -15088,6 +15328,12 @@
       <c r="M40" s="17" t="n">
         <v>53</v>
       </c>
+      <c r="N40" s="17" t="n">
+        <v>13</v>
+      </c>
+      <c r="O40" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="18" t="n">
@@ -15139,6 +15385,12 @@
       <c r="M41" s="20" t="n">
         <v>44</v>
       </c>
+      <c r="N41" s="20" t="n">
+        <v>19</v>
+      </c>
+      <c r="O41" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="15" t="n">
@@ -15190,6 +15442,12 @@
       <c r="M42" s="17" t="n">
         <v>42</v>
       </c>
+      <c r="N42" s="17" t="n">
+        <v>17</v>
+      </c>
+      <c r="O42" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="18" t="n">
@@ -15241,6 +15499,12 @@
       <c r="M43" s="20" t="n">
         <v>22</v>
       </c>
+      <c r="N43" s="20" t="n">
+        <v>14</v>
+      </c>
+      <c r="O43" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="15" t="n">
@@ -15292,6 +15556,12 @@
       <c r="M44" s="17" t="n">
         <v>37</v>
       </c>
+      <c r="N44" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="O44" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="18" t="n">
@@ -15343,6 +15613,12 @@
       <c r="M45" s="20" t="n">
         <v>26</v>
       </c>
+      <c r="N45" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="O45" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="15" t="n">
@@ -15394,6 +15670,12 @@
       <c r="M46" s="17" t="n">
         <v>51</v>
       </c>
+      <c r="N46" s="17" t="n">
+        <v>21</v>
+      </c>
+      <c r="O46" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="18" t="n">
@@ -15445,6 +15727,12 @@
       <c r="M47" s="20" t="n">
         <v>18</v>
       </c>
+      <c r="N47" s="20" t="n">
+        <v>8</v>
+      </c>
+      <c r="O47" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="15" t="n">
@@ -15496,6 +15784,12 @@
       <c r="M48" s="17" t="n">
         <v>38</v>
       </c>
+      <c r="N48" s="17" t="n">
+        <v>15</v>
+      </c>
+      <c r="O48" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="18" t="n">
@@ -15547,6 +15841,12 @@
       <c r="M49" s="20" t="n">
         <v>36</v>
       </c>
+      <c r="N49" s="20" t="n">
+        <v>9</v>
+      </c>
+      <c r="O49" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="15" t="n">
@@ -15598,6 +15898,12 @@
       <c r="M50" s="17" t="n">
         <v>119</v>
       </c>
+      <c r="N50" s="17" t="n">
+        <v>52</v>
+      </c>
+      <c r="O50" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="18" t="n">
@@ -15649,6 +15955,12 @@
       <c r="M51" s="20" t="n">
         <v>20</v>
       </c>
+      <c r="N51" s="20" t="n">
+        <v>9</v>
+      </c>
+      <c r="O51" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="15" t="n">
@@ -15700,6 +16012,12 @@
       <c r="M52" s="17" t="n">
         <v>27</v>
       </c>
+      <c r="N52" s="17" t="n">
+        <v>13</v>
+      </c>
+      <c r="O52" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="18" t="n">
@@ -15751,6 +16069,12 @@
       <c r="M53" s="20" t="n">
         <v>19</v>
       </c>
+      <c r="N53" s="20" t="n">
+        <v>12</v>
+      </c>
+      <c r="O53" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="15" t="n">
@@ -15802,6 +16126,12 @@
       <c r="M54" s="17" t="n">
         <v>85</v>
       </c>
+      <c r="N54" s="17" t="n">
+        <v>26</v>
+      </c>
+      <c r="O54" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="18" t="n">
@@ -15853,6 +16183,12 @@
       <c r="M55" s="20" t="n">
         <v>33</v>
       </c>
+      <c r="N55" s="20" t="n">
+        <v>14</v>
+      </c>
+      <c r="O55" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="15" t="n">
@@ -15904,6 +16240,12 @@
       <c r="M56" s="17" t="n">
         <v>0</v>
       </c>
+      <c r="N56" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="O56" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="18" t="n">
@@ -15955,6 +16297,12 @@
       <c r="M57" s="20" t="n">
         <v>32</v>
       </c>
+      <c r="N57" s="20" t="n">
+        <v>7</v>
+      </c>
+      <c r="O57" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="15" t="n">
@@ -16006,6 +16354,12 @@
       <c r="M58" s="17" t="n">
         <v>110</v>
       </c>
+      <c r="N58" s="17" t="n">
+        <v>39</v>
+      </c>
+      <c r="O58" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="18" t="n">
@@ -16057,6 +16411,12 @@
       <c r="M59" s="20" t="n">
         <v>58</v>
       </c>
+      <c r="N59" s="20" t="n">
+        <v>20</v>
+      </c>
+      <c r="O59" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="15" t="n">
@@ -16108,6 +16468,12 @@
       <c r="M60" s="17" t="n">
         <v>25</v>
       </c>
+      <c r="N60" s="17" t="n">
+        <v>5</v>
+      </c>
+      <c r="O60" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="18" t="n">
@@ -16159,6 +16525,12 @@
       <c r="M61" s="20" t="n">
         <v>0</v>
       </c>
+      <c r="N61" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="O61" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="15" t="n">
@@ -16210,6 +16582,12 @@
       <c r="M62" s="17" t="n">
         <v>27</v>
       </c>
+      <c r="N62" s="17" t="n">
+        <v>11</v>
+      </c>
+      <c r="O62" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="18" t="n">
@@ -16261,6 +16639,12 @@
       <c r="M63" s="20" t="n">
         <v>30</v>
       </c>
+      <c r="N63" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="O63" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="15" t="n">
@@ -16312,6 +16696,12 @@
       <c r="M64" s="17" t="n">
         <v>74</v>
       </c>
+      <c r="N64" s="17" t="n">
+        <v>26</v>
+      </c>
+      <c r="O64" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="18" t="n">
@@ -16363,6 +16753,12 @@
       <c r="M65" s="20" t="n">
         <v>46</v>
       </c>
+      <c r="N65" s="20" t="n">
+        <v>12</v>
+      </c>
+      <c r="O65" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="15" t="n">
@@ -16414,6 +16810,12 @@
       <c r="M66" s="17" t="n">
         <v>46</v>
       </c>
+      <c r="N66" s="17" t="n">
+        <v>10</v>
+      </c>
+      <c r="O66" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="18" t="n">
@@ -16465,6 +16867,12 @@
       <c r="M67" s="20" t="n">
         <v>44</v>
       </c>
+      <c r="N67" s="20" t="n">
+        <v>14</v>
+      </c>
+      <c r="O67" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="15" t="n">
@@ -16516,6 +16924,12 @@
       <c r="M68" s="17" t="n">
         <v>56</v>
       </c>
+      <c r="N68" s="17" t="n">
+        <v>19</v>
+      </c>
+      <c r="O68" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="18" t="n">
@@ -16567,6 +16981,12 @@
       <c r="M69" s="20" t="n">
         <v>21</v>
       </c>
+      <c r="N69" s="20" t="n">
+        <v>9</v>
+      </c>
+      <c r="O69" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="15" t="n">
@@ -16618,6 +17038,12 @@
       <c r="M70" s="17" t="n">
         <v>20</v>
       </c>
+      <c r="N70" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="O70" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="18" t="n">
@@ -16669,6 +17095,12 @@
       <c r="M71" s="20" t="n">
         <v>51</v>
       </c>
+      <c r="N71" s="20" t="n">
+        <v>18</v>
+      </c>
+      <c r="O71" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="15" t="n">
@@ -16720,6 +17152,12 @@
       <c r="M72" s="17" t="n">
         <v>54</v>
       </c>
+      <c r="N72" s="17" t="n">
+        <v>20</v>
+      </c>
+      <c r="O72" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="18" t="n">
@@ -16771,6 +17209,12 @@
       <c r="M73" s="20" t="n">
         <v>56</v>
       </c>
+      <c r="N73" s="20" t="n">
+        <v>23</v>
+      </c>
+      <c r="O73" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="15" t="n">
@@ -16822,6 +17266,12 @@
       <c r="M74" s="17" t="n">
         <v>12</v>
       </c>
+      <c r="N74" s="17" t="n">
+        <v>12</v>
+      </c>
+      <c r="O74" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="18" t="n">
@@ -16873,6 +17323,12 @@
       <c r="M75" s="20" t="n">
         <v>17</v>
       </c>
+      <c r="N75" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="O75" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="15" t="n">
@@ -16924,6 +17380,12 @@
       <c r="M76" s="17" t="n">
         <v>0</v>
       </c>
+      <c r="N76" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="O76" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="18" t="n">
@@ -16975,6 +17437,12 @@
       <c r="M77" s="20" t="n">
         <v>24</v>
       </c>
+      <c r="N77" s="20" t="n">
+        <v>8</v>
+      </c>
+      <c r="O77" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="15" t="n">
@@ -17026,6 +17494,12 @@
       <c r="M78" s="17" t="n">
         <v>19</v>
       </c>
+      <c r="N78" s="17" t="n">
+        <v>9</v>
+      </c>
+      <c r="O78" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="18" t="n">
@@ -17077,6 +17551,12 @@
       <c r="M79" s="20" t="n">
         <v>27</v>
       </c>
+      <c r="N79" s="20" t="n">
+        <v>15</v>
+      </c>
+      <c r="O79" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="15" t="n">
@@ -17128,6 +17608,12 @@
       <c r="M80" s="17" t="n">
         <v>10</v>
       </c>
+      <c r="N80" s="17" t="n">
+        <v>7</v>
+      </c>
+      <c r="O80" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="18" t="n">
@@ -17179,6 +17665,12 @@
       <c r="M81" s="20" t="n">
         <v>46</v>
       </c>
+      <c r="N81" s="20" t="n">
+        <v>19</v>
+      </c>
+      <c r="O81" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="15" t="n">
@@ -17230,6 +17722,12 @@
       <c r="M82" s="17" t="n">
         <v>40</v>
       </c>
+      <c r="N82" s="17" t="n">
+        <v>16</v>
+      </c>
+      <c r="O82" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="18" t="n">
@@ -17281,6 +17779,12 @@
       <c r="M83" s="20" t="n">
         <v>16</v>
       </c>
+      <c r="N83" s="20" t="n">
+        <v>7</v>
+      </c>
+      <c r="O83" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="15" t="n">
@@ -17332,6 +17836,12 @@
       <c r="M84" s="17" t="n">
         <v>67</v>
       </c>
+      <c r="N84" s="17" t="n">
+        <v>21</v>
+      </c>
+      <c r="O84" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="18" t="n">
@@ -17383,6 +17893,12 @@
       <c r="M85" s="20" t="n">
         <v>0</v>
       </c>
+      <c r="N85" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="O85" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="15" t="n">
@@ -17434,6 +17950,12 @@
       <c r="M86" s="17" t="n">
         <v>25</v>
       </c>
+      <c r="N86" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="O86" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="18" t="n">
@@ -17485,6 +18007,12 @@
       <c r="M87" s="20" t="n">
         <v>3</v>
       </c>
+      <c r="N87" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="O87" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="15" t="n">
@@ -17536,6 +18064,12 @@
       <c r="M88" s="17" t="n">
         <v>3</v>
       </c>
+      <c r="N88" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="O88" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="18" t="n">
@@ -17587,6 +18121,12 @@
       <c r="M89" s="20" t="n">
         <v>21</v>
       </c>
+      <c r="N89" s="20" t="n">
+        <v>9</v>
+      </c>
+      <c r="O89" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="15" t="n">
@@ -17638,6 +18178,12 @@
       <c r="M90" s="17" t="n">
         <v>48</v>
       </c>
+      <c r="N90" s="17" t="n">
+        <v>20</v>
+      </c>
+      <c r="O90" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="18" t="n">
@@ -17689,6 +18235,12 @@
       <c r="M91" s="20" t="n">
         <v>21</v>
       </c>
+      <c r="N91" s="20" t="n">
+        <v>11</v>
+      </c>
+      <c r="O91" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="15" t="n">
@@ -17740,6 +18292,12 @@
       <c r="M92" s="17" t="n">
         <v>64</v>
       </c>
+      <c r="N92" s="17" t="n">
+        <v>16</v>
+      </c>
+      <c r="O92" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="18" t="n">
@@ -17791,6 +18349,12 @@
       <c r="M93" s="20" t="n">
         <v>79</v>
       </c>
+      <c r="N93" s="20" t="n">
+        <v>23</v>
+      </c>
+      <c r="O93" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="15" t="n">
@@ -17842,6 +18406,12 @@
       <c r="M94" s="17" t="n">
         <v>44</v>
       </c>
+      <c r="N94" s="17" t="n">
+        <v>12</v>
+      </c>
+      <c r="O94" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="18" t="n">
@@ -17893,6 +18463,12 @@
       <c r="M95" s="20" t="n">
         <v>79</v>
       </c>
+      <c r="N95" s="20" t="n">
+        <v>31</v>
+      </c>
+      <c r="O95" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="15" t="n">
@@ -17944,6 +18520,12 @@
       <c r="M96" s="17" t="n">
         <v>65</v>
       </c>
+      <c r="N96" s="17" t="n">
+        <v>24</v>
+      </c>
+      <c r="O96" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="18" t="n">
@@ -17995,6 +18577,12 @@
       <c r="M97" s="20" t="n">
         <v>21</v>
       </c>
+      <c r="N97" s="20" t="n">
+        <v>9</v>
+      </c>
+      <c r="O97" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="15" t="n">
@@ -18046,6 +18634,12 @@
       <c r="M98" s="17" t="n">
         <v>51</v>
       </c>
+      <c r="N98" s="17" t="n">
+        <v>18</v>
+      </c>
+      <c r="O98" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="18" t="n">
@@ -18097,6 +18691,12 @@
       <c r="M99" s="20" t="n">
         <v>75</v>
       </c>
+      <c r="N99" s="20" t="n">
+        <v>32</v>
+      </c>
+      <c r="O99" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="15" t="n">
@@ -18148,6 +18748,12 @@
       <c r="M100" s="17" t="n">
         <v>76</v>
       </c>
+      <c r="N100" s="17" t="n">
+        <v>19</v>
+      </c>
+      <c r="O100" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="18" t="n">
@@ -18199,6 +18805,12 @@
       <c r="M101" s="20" t="n">
         <v>27</v>
       </c>
+      <c r="N101" s="20" t="n">
+        <v>16</v>
+      </c>
+      <c r="O101" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="15" t="n">
@@ -18250,6 +18862,12 @@
       <c r="M102" s="17" t="n">
         <v>28</v>
       </c>
+      <c r="N102" s="17" t="n">
+        <v>16</v>
+      </c>
+      <c r="O102" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="18" t="n">
@@ -18301,6 +18919,12 @@
       <c r="M103" s="20" t="n">
         <v>28</v>
       </c>
+      <c r="N103" s="20" t="n">
+        <v>15</v>
+      </c>
+      <c r="O103" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="15" t="n">
@@ -18352,6 +18976,12 @@
       <c r="M104" s="17" t="n">
         <v>27</v>
       </c>
+      <c r="N104" s="17" t="n">
+        <v>15</v>
+      </c>
+      <c r="O104" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="18" t="n">
@@ -18403,6 +19033,12 @@
       <c r="M105" s="20" t="n">
         <v>28</v>
       </c>
+      <c r="N105" s="20" t="n">
+        <v>10</v>
+      </c>
+      <c r="O105" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="15" t="n">
@@ -18454,6 +19090,12 @@
       <c r="M106" s="17" t="n">
         <v>32</v>
       </c>
+      <c r="N106" s="17" t="n">
+        <v>9</v>
+      </c>
+      <c r="O106" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="18" t="n">
@@ -18505,6 +19147,12 @@
       <c r="M107" s="20" t="n">
         <v>72</v>
       </c>
+      <c r="N107" s="20" t="n">
+        <v>25</v>
+      </c>
+      <c r="O107" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="15" t="n">
@@ -18556,6 +19204,12 @@
       <c r="M108" s="17" t="n">
         <v>35</v>
       </c>
+      <c r="N108" s="17" t="n">
+        <v>12</v>
+      </c>
+      <c r="O108" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="18" t="n">
@@ -18607,6 +19261,12 @@
       <c r="M109" s="20" t="n">
         <v>72</v>
       </c>
+      <c r="N109" s="20" t="n">
+        <v>34</v>
+      </c>
+      <c r="O109" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="15" t="n">
@@ -18658,6 +19318,12 @@
       <c r="M110" s="17" t="n">
         <v>18</v>
       </c>
+      <c r="N110" s="17" t="n">
+        <v>10</v>
+      </c>
+      <c r="O110" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="18" t="n">
@@ -18709,6 +19375,12 @@
       <c r="M111" s="20" t="n">
         <v>59</v>
       </c>
+      <c r="N111" s="20" t="n">
+        <v>25</v>
+      </c>
+      <c r="O111" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="15" t="n">
@@ -18760,6 +19432,12 @@
       <c r="M112" s="17" t="n">
         <v>19</v>
       </c>
+      <c r="N112" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="O112" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="18" t="n">
@@ -18811,6 +19489,12 @@
       <c r="M113" s="20" t="n">
         <v>53</v>
       </c>
+      <c r="N113" s="20" t="n">
+        <v>22</v>
+      </c>
+      <c r="O113" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="15" t="n">
@@ -18862,6 +19546,12 @@
       <c r="M114" s="17" t="n">
         <v>43</v>
       </c>
+      <c r="N114" s="17" t="n">
+        <v>16</v>
+      </c>
+      <c r="O114" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="18" t="n">
@@ -18913,6 +19603,12 @@
       <c r="M115" s="20" t="n">
         <v>39</v>
       </c>
+      <c r="N115" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="O115" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="15" t="n">
@@ -18964,6 +19660,12 @@
       <c r="M116" s="17" t="n">
         <v>35</v>
       </c>
+      <c r="N116" s="17" t="n">
+        <v>14</v>
+      </c>
+      <c r="O116" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="18" t="n">
@@ -19015,6 +19717,12 @@
       <c r="M117" s="20" t="n">
         <v>19</v>
       </c>
+      <c r="N117" s="20" t="n">
+        <v>9</v>
+      </c>
+      <c r="O117" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="15" t="n">
@@ -19066,6 +19774,12 @@
       <c r="M118" s="17" t="n">
         <v>20</v>
       </c>
+      <c r="N118" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="O118" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="18" t="n">
@@ -19117,6 +19831,12 @@
       <c r="M119" s="20" t="n">
         <v>20</v>
       </c>
+      <c r="N119" s="20" t="n">
+        <v>9</v>
+      </c>
+      <c r="O119" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="15" t="n">
@@ -19168,6 +19888,12 @@
       <c r="M120" s="17" t="n">
         <v>66</v>
       </c>
+      <c r="N120" s="17" t="n">
+        <v>28</v>
+      </c>
+      <c r="O120" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="18" t="n">
@@ -19219,6 +19945,12 @@
       <c r="M121" s="20" t="n">
         <v>39</v>
       </c>
+      <c r="N121" s="20" t="n">
+        <v>13</v>
+      </c>
+      <c r="O121" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="15" t="n">
@@ -19270,6 +20002,12 @@
       <c r="M122" s="17" t="n">
         <v>37</v>
       </c>
+      <c r="N122" s="17" t="n">
+        <v>15</v>
+      </c>
+      <c r="O122" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="18" t="n">
@@ -19321,6 +20059,12 @@
       <c r="M123" s="20" t="n">
         <v>50</v>
       </c>
+      <c r="N123" s="20" t="n">
+        <v>25</v>
+      </c>
+      <c r="O123" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="15" t="n">
@@ -19372,6 +20116,12 @@
       <c r="M124" s="17" t="n">
         <v>39</v>
       </c>
+      <c r="N124" s="17" t="n">
+        <v>14</v>
+      </c>
+      <c r="O124" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="18" t="n">
@@ -19423,6 +20173,12 @@
       <c r="M125" s="20" t="n">
         <v>40</v>
       </c>
+      <c r="N125" s="20" t="n">
+        <v>20</v>
+      </c>
+      <c r="O125" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="15" t="n">
@@ -19474,6 +20230,12 @@
       <c r="M126" s="17" t="n">
         <v>44</v>
       </c>
+      <c r="N126" s="17" t="n">
+        <v>21</v>
+      </c>
+      <c r="O126" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="18" t="n">
@@ -19525,6 +20287,12 @@
       <c r="M127" s="20" t="n">
         <v>35</v>
       </c>
+      <c r="N127" s="20" t="n">
+        <v>15</v>
+      </c>
+      <c r="O127" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="15" t="n">
@@ -19576,6 +20344,12 @@
       <c r="M128" s="17" t="n">
         <v>90</v>
       </c>
+      <c r="N128" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="O128" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="18" t="n">
@@ -19627,6 +20401,12 @@
       <c r="M129" s="20" t="n">
         <v>72</v>
       </c>
+      <c r="N129" s="20" t="n">
+        <v>28</v>
+      </c>
+      <c r="O129" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="15" t="n">
@@ -19678,6 +20458,12 @@
       <c r="M130" s="17" t="n">
         <v>23</v>
       </c>
+      <c r="N130" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="O130" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="18" t="n">
@@ -19729,6 +20515,12 @@
       <c r="M131" s="20" t="n">
         <v>18</v>
       </c>
+      <c r="N131" s="20" t="n">
+        <v>10</v>
+      </c>
+      <c r="O131" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="15" t="n">
@@ -19780,6 +20572,12 @@
       <c r="M132" s="17" t="n">
         <v>17</v>
       </c>
+      <c r="N132" s="17" t="n">
+        <v>7</v>
+      </c>
+      <c r="O132" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="18" t="n">
@@ -19831,6 +20629,12 @@
       <c r="M133" s="20" t="n">
         <v>41</v>
       </c>
+      <c r="N133" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="O133" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="15" t="n">
@@ -19882,6 +20686,12 @@
       <c r="M134" s="17" t="n">
         <v>83</v>
       </c>
+      <c r="N134" s="17" t="n">
+        <v>33</v>
+      </c>
+      <c r="O134" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="18" t="n">
@@ -19933,6 +20743,12 @@
       <c r="M135" s="20" t="n">
         <v>65</v>
       </c>
+      <c r="N135" s="20" t="n">
+        <v>24</v>
+      </c>
+      <c r="O135" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="15" t="n">
@@ -19984,6 +20800,12 @@
       <c r="M136" s="17" t="n">
         <v>19</v>
       </c>
+      <c r="N136" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="O136" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="18" t="n">
@@ -20035,6 +20857,12 @@
       <c r="M137" s="20" t="n">
         <v>82</v>
       </c>
+      <c r="N137" s="20" t="n">
+        <v>38</v>
+      </c>
+      <c r="O137" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="15" t="n">
@@ -20086,6 +20914,12 @@
       <c r="M138" s="17" t="n">
         <v>43</v>
       </c>
+      <c r="N138" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="O138" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="18" t="n">
@@ -20137,6 +20971,12 @@
       <c r="M139" s="20" t="n">
         <v>48</v>
       </c>
+      <c r="N139" s="20" t="n">
+        <v>21</v>
+      </c>
+      <c r="O139" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="15" t="n">
@@ -20188,6 +21028,12 @@
       <c r="M140" s="17" t="n">
         <v>25</v>
       </c>
+      <c r="N140" s="17" t="n">
+        <v>12</v>
+      </c>
+      <c r="O140" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="18" t="n">
@@ -20239,6 +21085,12 @@
       <c r="M141" s="20" t="n">
         <v>49</v>
       </c>
+      <c r="N141" s="20" t="n">
+        <v>18</v>
+      </c>
+      <c r="O141" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="15" t="n">
@@ -20290,6 +21142,12 @@
       <c r="M142" s="17" t="n">
         <v>41</v>
       </c>
+      <c r="N142" s="17" t="n">
+        <v>17</v>
+      </c>
+      <c r="O142" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="18" t="n">
@@ -20341,6 +21199,12 @@
       <c r="M143" s="20" t="n">
         <v>48</v>
       </c>
+      <c r="N143" s="20" t="n">
+        <v>16</v>
+      </c>
+      <c r="O143" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="15" t="n">
@@ -20392,6 +21256,12 @@
       <c r="M144" s="17" t="n">
         <v>33</v>
       </c>
+      <c r="N144" s="17" t="n">
+        <v>11</v>
+      </c>
+      <c r="O144" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="18" t="n">
@@ -20443,6 +21313,12 @@
       <c r="M145" s="20" t="n">
         <v>26</v>
       </c>
+      <c r="N145" s="20" t="n">
+        <v>15</v>
+      </c>
+      <c r="O145" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="15" t="n">
@@ -20494,6 +21370,12 @@
       <c r="M146" s="17" t="n">
         <v>57</v>
       </c>
+      <c r="N146" s="17" t="n">
+        <v>16</v>
+      </c>
+      <c r="O146" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="18" t="n">
@@ -20545,6 +21427,12 @@
       <c r="M147" s="20" t="n">
         <v>25</v>
       </c>
+      <c r="N147" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="O147" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="15" t="n">
@@ -20596,6 +21484,12 @@
       <c r="M148" s="17" t="n">
         <v>119</v>
       </c>
+      <c r="N148" s="17" t="n">
+        <v>50</v>
+      </c>
+      <c r="O148" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="18" t="n">
@@ -20647,6 +21541,12 @@
       <c r="M149" s="20" t="n">
         <v>37</v>
       </c>
+      <c r="N149" s="20" t="n">
+        <v>16</v>
+      </c>
+      <c r="O149" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="15" t="n">
@@ -20698,6 +21598,12 @@
       <c r="M150" s="17" t="n">
         <v>26</v>
       </c>
+      <c r="N150" s="17" t="n">
+        <v>13</v>
+      </c>
+      <c r="O150" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="18" t="n">
@@ -20749,6 +21655,12 @@
       <c r="M151" s="20" t="n">
         <v>29</v>
       </c>
+      <c r="N151" s="20" t="n">
+        <v>17</v>
+      </c>
+      <c r="O151" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="15" t="n">
@@ -20800,6 +21712,12 @@
       <c r="M152" s="17" t="n">
         <v>0</v>
       </c>
+      <c r="N152" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="O152" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="18" t="n">
@@ -20851,6 +21769,12 @@
       <c r="M153" s="20" t="n">
         <v>60</v>
       </c>
+      <c r="N153" s="20" t="n">
+        <v>27</v>
+      </c>
+      <c r="O153" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="15" t="n">
@@ -20902,6 +21826,12 @@
       <c r="M154" s="17" t="n">
         <v>42</v>
       </c>
+      <c r="N154" s="17" t="n">
+        <v>14</v>
+      </c>
+      <c r="O154" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="18" t="n">
@@ -20953,6 +21883,12 @@
       <c r="M155" s="20" t="n">
         <v>19</v>
       </c>
+      <c r="N155" s="20" t="n">
+        <v>8</v>
+      </c>
+      <c r="O155" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="15" t="n">
@@ -21004,6 +21940,12 @@
       <c r="M156" s="17" t="n">
         <v>2</v>
       </c>
+      <c r="N156" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="O156" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="18" t="n">
@@ -21055,6 +21997,12 @@
       <c r="M157" s="20" t="n">
         <v>59</v>
       </c>
+      <c r="N157" s="20" t="n">
+        <v>30</v>
+      </c>
+      <c r="O157" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="15" t="n">
@@ -21106,6 +22054,12 @@
       <c r="M158" s="17" t="n">
         <v>16</v>
       </c>
+      <c r="N158" s="17" t="n">
+        <v>7</v>
+      </c>
+      <c r="O158" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="18" t="n">
@@ -21157,6 +22111,12 @@
       <c r="M159" s="20" t="n">
         <v>20</v>
       </c>
+      <c r="N159" s="20" t="n">
+        <v>20</v>
+      </c>
+      <c r="O159" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="15" t="n">
@@ -21208,6 +22168,12 @@
       <c r="M160" s="17" t="n">
         <v>63</v>
       </c>
+      <c r="N160" s="17" t="n">
+        <v>25</v>
+      </c>
+      <c r="O160" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="18" t="n">
@@ -21259,6 +22225,12 @@
       <c r="M161" s="20" t="n">
         <v>36</v>
       </c>
+      <c r="N161" s="20" t="n">
+        <v>17</v>
+      </c>
+      <c r="O161" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="15" t="n">
@@ -21310,6 +22282,12 @@
       <c r="M162" s="17" t="n">
         <v>61</v>
       </c>
+      <c r="N162" s="17" t="n">
+        <v>12</v>
+      </c>
+      <c r="O162" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="18" t="n">
@@ -21361,6 +22339,12 @@
       <c r="M163" s="20" t="n">
         <v>40</v>
       </c>
+      <c r="N163" s="20" t="n">
+        <v>16</v>
+      </c>
+      <c r="O163" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="15" t="n">
@@ -21412,6 +22396,12 @@
       <c r="M164" s="17" t="n">
         <v>31</v>
       </c>
+      <c r="N164" s="17" t="n">
+        <v>13</v>
+      </c>
+      <c r="O164" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="18" t="n">
@@ -21463,6 +22453,12 @@
       <c r="M165" s="20" t="n">
         <v>29</v>
       </c>
+      <c r="N165" s="20" t="n">
+        <v>11</v>
+      </c>
+      <c r="O165" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="166">
       <c r="A166" s="15" t="n">
@@ -21514,6 +22510,12 @@
       <c r="M166" s="17" t="n">
         <v>23</v>
       </c>
+      <c r="N166" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="O166" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="167">
       <c r="A167" s="18" t="n">
@@ -21565,6 +22567,12 @@
       <c r="M167" s="20" t="n">
         <v>9</v>
       </c>
+      <c r="N167" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="O167" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="168">
       <c r="A168" s="15" t="n">
@@ -21616,6 +22624,12 @@
       <c r="M168" s="17" t="n">
         <v>31</v>
       </c>
+      <c r="N168" s="17" t="n">
+        <v>12</v>
+      </c>
+      <c r="O168" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="169">
       <c r="A169" s="18" t="n">
@@ -21667,6 +22681,12 @@
       <c r="M169" s="20" t="n">
         <v>20</v>
       </c>
+      <c r="N169" s="20" t="n">
+        <v>9</v>
+      </c>
+      <c r="O169" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="170">
       <c r="A170" s="15" t="n">
@@ -21718,6 +22738,12 @@
       <c r="M170" s="17" t="n">
         <v>39</v>
       </c>
+      <c r="N170" s="17" t="n">
+        <v>13</v>
+      </c>
+      <c r="O170" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="171">
       <c r="A171" s="18" t="n">
@@ -21769,6 +22795,12 @@
       <c r="M171" s="20" t="n">
         <v>44</v>
       </c>
+      <c r="N171" s="20" t="n">
+        <v>19</v>
+      </c>
+      <c r="O171" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="172">
       <c r="A172" s="15" t="n">
@@ -21820,6 +22852,12 @@
       <c r="M172" s="17" t="n">
         <v>54</v>
       </c>
+      <c r="N172" s="17" t="n">
+        <v>10</v>
+      </c>
+      <c r="O172" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="173">
       <c r="A173" s="18" t="n">
@@ -21871,6 +22909,12 @@
       <c r="M173" s="20" t="n">
         <v>0</v>
       </c>
+      <c r="N173" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="O173" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="174">
       <c r="A174" s="15" t="n">
@@ -21922,6 +22966,12 @@
       <c r="M174" s="17" t="n">
         <v>61</v>
       </c>
+      <c r="N174" s="17" t="n">
+        <v>23</v>
+      </c>
+      <c r="O174" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="175">
       <c r="A175" s="18" t="n">
@@ -21973,6 +23023,12 @@
       <c r="M175" s="20" t="n">
         <v>91</v>
       </c>
+      <c r="N175" s="20" t="n">
+        <v>23</v>
+      </c>
+      <c r="O175" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="176">
       <c r="A176" s="15" t="n">
@@ -22024,6 +23080,12 @@
       <c r="M176" s="17" t="n">
         <v>29</v>
       </c>
+      <c r="N176" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="O176" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="177">
       <c r="A177" s="18" t="n">
@@ -22075,6 +23137,12 @@
       <c r="M177" s="20" t="n">
         <v>52</v>
       </c>
+      <c r="N177" s="20" t="n">
+        <v>15</v>
+      </c>
+      <c r="O177" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="178">
       <c r="A178" s="15" t="n">
@@ -22126,6 +23194,12 @@
       <c r="M178" s="17" t="n">
         <v>53</v>
       </c>
+      <c r="N178" s="17" t="n">
+        <v>20</v>
+      </c>
+      <c r="O178" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="179">
       <c r="A179" s="18" t="n">
@@ -22177,6 +23251,12 @@
       <c r="M179" s="20" t="n">
         <v>95</v>
       </c>
+      <c r="N179" s="20" t="n">
+        <v>33</v>
+      </c>
+      <c r="O179" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="180">
       <c r="A180" s="15" t="n">
@@ -22228,6 +23308,12 @@
       <c r="M180" s="17" t="n">
         <v>12</v>
       </c>
+      <c r="N180" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="O180" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="181">
       <c r="A181" s="18" t="n">
@@ -22279,6 +23365,12 @@
       <c r="M181" s="20" t="n">
         <v>45</v>
       </c>
+      <c r="N181" s="20" t="n">
+        <v>21</v>
+      </c>
+      <c r="O181" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="182">
       <c r="A182" s="15" t="n">
@@ -22330,6 +23422,12 @@
       <c r="M182" s="17" t="n">
         <v>48</v>
       </c>
+      <c r="N182" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="O182" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="183">
       <c r="A183" s="18" t="n">
@@ -22381,6 +23479,12 @@
       <c r="M183" s="20" t="n">
         <v>24</v>
       </c>
+      <c r="N183" s="20" t="n">
+        <v>11</v>
+      </c>
+      <c r="O183" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="184">
       <c r="A184" s="15" t="n">
@@ -22432,6 +23536,12 @@
       <c r="M184" s="17" t="n">
         <v>107</v>
       </c>
+      <c r="N184" s="17" t="n">
+        <v>46</v>
+      </c>
+      <c r="O184" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="185">
       <c r="A185" s="18" t="n">
@@ -22483,6 +23593,12 @@
       <c r="M185" s="20" t="n">
         <v>51</v>
       </c>
+      <c r="N185" s="20" t="n">
+        <v>21</v>
+      </c>
+      <c r="O185" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="186">
       <c r="A186" s="15" t="n">
@@ -22534,6 +23650,12 @@
       <c r="M186" s="17" t="n">
         <v>20</v>
       </c>
+      <c r="N186" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="O186" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="187">
       <c r="A187" s="18" t="n">
@@ -22585,6 +23707,12 @@
       <c r="M187" s="20" t="n">
         <v>39</v>
       </c>
+      <c r="N187" s="20" t="n">
+        <v>16</v>
+      </c>
+      <c r="O187" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="188">
       <c r="A188" s="15" t="n">
@@ -22636,6 +23764,12 @@
       <c r="M188" s="17" t="n">
         <v>64</v>
       </c>
+      <c r="N188" s="17" t="n">
+        <v>25</v>
+      </c>
+      <c r="O188" s="17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="189">
       <c r="A189" s="18" t="n">
@@ -22687,6 +23821,12 @@
       <c r="M189" s="20" t="n">
         <v>28</v>
       </c>
+      <c r="N189" s="20" t="n">
+        <v>9</v>
+      </c>
+      <c r="O189" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="190">
       <c r="A190" s="15" t="n">
@@ -22737,6 +23877,12 @@
       </c>
       <c r="M190" s="17" t="n">
         <v>99</v>
+      </c>
+      <c r="N190" s="17" t="n">
+        <v>41</v>
+      </c>
+      <c r="O190" s="17" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>